<commit_message>
Simplify DECAT to an English-only runnable source package
</commit_message>
<xml_diff>
--- a/data/DECAT_Dataset_with_References.xlsx
+++ b/data/DECAT_Dataset_with_References.xlsx
@@ -4,16 +4,14 @@
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\个人资料\科研、科创团队、大创\科研\科研代码\outputs\01a0eccd-458e-7b22-9054-be5d4812b798\"/>
-    </mc:Choice>
+    <mc:Choice Requires="x15"/>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF5B17EB-9B75-4278-A1ED-CFEF51724FCE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="原始数据" sheetId="1" r:id="rId1"/>
+    <sheet name="Data" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
@@ -3650,7 +3648,7 @@
     </font>
     <font>
       <sz val="9"/>
-      <name val="宋体"/>
+      <name val="SimSun"/>
       <family val="3"/>
       <charset val="134"/>
     </font>
@@ -3744,7 +3742,7 @@
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>

</xml_diff>